<commit_message>
Refactor: tres archivos principales
</commit_message>
<xml_diff>
--- a/2026/indicadores_diarios.xlsx
+++ b/2026/indicadores_diarios.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M466"/>
+  <dimension ref="A1:M497"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5917,10 +5917,10 @@
         <v>46075</v>
       </c>
       <c r="C138" t="n">
-        <v>0.4884690438100637</v>
+        <v>0.4880483656479648</v>
       </c>
       <c r="D138" t="n">
-        <v>2.047212638491867</v>
+        <v>2.048977253867728</v>
       </c>
       <c r="E138" t="n">
         <v>0.5240486058818987</v>
@@ -5932,22 +5932,22 @@
         <v>0.6766304263228504</v>
       </c>
       <c r="H138" t="n">
-        <v>0.7510566905452363</v>
+        <v>0.7939108710726334</v>
       </c>
       <c r="I138" t="n">
-        <v>11.47504308866921</v>
+        <v>11.37692204308833</v>
       </c>
       <c r="J138" t="n">
-        <v>0.06018491236816401</v>
+        <v>0.05967028192328237</v>
       </c>
       <c r="K138" t="n">
-        <v>0.1467516618445535</v>
+        <v>0.1372188134029763</v>
       </c>
       <c r="L138" t="n">
-        <v>0.9572219696969696</v>
+        <v>0.9533465277777777</v>
       </c>
       <c r="M138" t="n">
-        <v>2.194096515151515</v>
+        <v>2.190045972222222</v>
       </c>
     </row>
     <row r="139">
@@ -6304,22 +6304,22 @@
         <v>46084</v>
       </c>
       <c r="C147" t="n">
-        <v>0.6416792501949651</v>
+        <v>0.6416837028942034</v>
       </c>
       <c r="D147" t="n">
-        <v>1.558410996921225</v>
+        <v>1.558400182971256</v>
       </c>
       <c r="E147" t="n">
-        <v>0.7859887845195</v>
+        <v>0.7859954635683575</v>
       </c>
       <c r="F147" t="n">
-        <v>0.1624553957428684</v>
+        <v>0.1624617720011293</v>
       </c>
       <c r="G147" t="n">
-        <v>0.7621554007055411</v>
+        <v>0.7621489242392074</v>
       </c>
       <c r="H147" t="n">
-        <v>0.4491923911633576</v>
+        <v>0.4491885741210641</v>
       </c>
       <c r="I147" t="n">
         <v>15.0745913601201</v>
@@ -6328,13 +6328,13 @@
         <v>0.0848672472820973</v>
       </c>
       <c r="K147" t="n">
-        <v>0.3265585028568002</v>
+        <v>0.3265348510808735</v>
       </c>
       <c r="L147" t="n">
-        <v>0.9809397294945921</v>
+        <v>0.9809379793103622</v>
       </c>
       <c r="M147" t="n">
-        <v>1.670407226098743</v>
+        <v>1.670383577118148</v>
       </c>
     </row>
     <row r="148">
@@ -13399,37 +13399,37 @@
         <v>46063</v>
       </c>
       <c r="C312" t="n">
-        <v>0.2512088189349099</v>
+        <v>0.2348447464332972</v>
       </c>
       <c r="D312" t="n">
-        <v>3.980751966590423</v>
+        <v>4.258132298837817</v>
       </c>
       <c r="E312" t="n">
-        <v>0.3309039587400608</v>
+        <v>0.3248925986214463</v>
       </c>
       <c r="F312" t="n">
-        <v>0.8252660027593705</v>
+        <v>0.8336855052449234</v>
       </c>
       <c r="G312" t="n">
-        <v>0.1023829995555783</v>
+        <v>0.1252858880483509</v>
       </c>
       <c r="H312" t="n">
-        <v>0.2774779113378196</v>
+        <v>0.1685142791473397</v>
       </c>
       <c r="I312" t="n">
-        <v>5.52789004922097</v>
+        <v>5.529194647269979</v>
       </c>
       <c r="J312" t="n">
-        <v>0.009219337570833213</v>
+        <v>0.009221513361180159</v>
       </c>
       <c r="K312" t="n">
-        <v>0.3064934951074728</v>
+        <v>0.3066899084543456</v>
       </c>
       <c r="L312" t="n">
-        <v>0.829881926486832</v>
+        <v>0.8348972222222223</v>
       </c>
       <c r="M312" t="n">
-        <v>1.538729526996491</v>
+        <v>1.540506319444444</v>
       </c>
     </row>
     <row r="313">
@@ -13442,37 +13442,37 @@
         <v>46064</v>
       </c>
       <c r="C313" t="n">
-        <v>0.2389410283847887</v>
+        <v>0.2259529920959361</v>
       </c>
       <c r="D313" t="n">
-        <v>4.185133071368589</v>
+        <v>4.42569930463862</v>
       </c>
       <c r="E313" t="n">
-        <v>0.320981885141168</v>
+        <v>0.315601709119364</v>
       </c>
       <c r="F313" t="n">
-        <v>0.9533899959045408</v>
+        <v>0.9836805453444291</v>
       </c>
       <c r="G313" t="n">
-        <v>0.112815841510312</v>
+        <v>0.1147390537992032</v>
       </c>
       <c r="H313" t="n">
-        <v>0.2332197495790365</v>
+        <v>0.1478304986980745</v>
       </c>
       <c r="I313" t="n">
-        <v>5.388906760286241</v>
+        <v>5.382336380633471</v>
       </c>
       <c r="J313" t="n">
-        <v>0.009987350433454972</v>
+        <v>0.009975173439680159</v>
       </c>
       <c r="K313" t="n">
-        <v>0.3113976184634992</v>
+        <v>0.313288396379262</v>
       </c>
       <c r="L313" t="n">
-        <v>0.8277226947072535</v>
+        <v>0.8329221153846155</v>
       </c>
       <c r="M313" t="n">
-        <v>1.492125374078536</v>
+        <v>1.489677200854701</v>
       </c>
     </row>
     <row r="314">
@@ -13485,22 +13485,22 @@
         <v>46065</v>
       </c>
       <c r="C314" t="n">
-        <v>0.2778490836313499</v>
+        <v>0.2527799720812597</v>
       </c>
       <c r="D314" t="n">
-        <v>3.599076113300412</v>
+        <v>3.956009614869867</v>
       </c>
       <c r="E314" t="n">
-        <v>0.3594430552503931</v>
+        <v>0.3578298670109216</v>
       </c>
       <c r="F314" t="n">
-        <v>1.000236333557291</v>
+        <v>1.00730823949156</v>
       </c>
       <c r="G314" t="n">
-        <v>0.08877741970186846</v>
+        <v>0.08366986846714718</v>
       </c>
       <c r="H314" t="n">
-        <v>0.2541392182689476</v>
+        <v>0.119275069402279</v>
       </c>
       <c r="I314" t="n">
         <v>6.064051209679804</v>
@@ -13509,13 +13509,13 @@
         <v>0.0107405474715</v>
       </c>
       <c r="K314" t="n">
-        <v>0.2757483525880827</v>
+        <v>0.2760656253440139</v>
       </c>
       <c r="L314" t="n">
-        <v>0.8463191978783662</v>
+        <v>0.8516548611111111</v>
       </c>
       <c r="M314" t="n">
-        <v>1.560151250118291</v>
+        <v>1.548991597222222</v>
       </c>
     </row>
     <row r="315">
@@ -13528,22 +13528,22 @@
         <v>46066</v>
       </c>
       <c r="C315" t="n">
-        <v>0.3859538116826756</v>
+        <v>0.3883532575617983</v>
       </c>
       <c r="D315" t="n">
-        <v>2.590983609256805</v>
+        <v>2.574975181818504</v>
       </c>
       <c r="E315" t="n">
-        <v>0.5327940585072275</v>
+        <v>0.523075201051505</v>
       </c>
       <c r="F315" t="n">
-        <v>0.5217583530792915</v>
+        <v>0.5469741264224893</v>
       </c>
       <c r="G315" t="n">
-        <v>0.182444905628571</v>
+        <v>0.1858347739070946</v>
       </c>
       <c r="H315" t="n">
-        <v>0.1731875882627166</v>
+        <v>0.2273274862645923</v>
       </c>
       <c r="I315" t="n">
         <v>9.249706206962099</v>
@@ -13552,13 +13552,13 @@
         <v>0.005790295541812793</v>
       </c>
       <c r="K315" t="n">
-        <v>0.2910021932197582</v>
+        <v>0.2904220657668427</v>
       </c>
       <c r="L315" t="n">
-        <v>0.8550704365079365</v>
+        <v>0.8556389190821255</v>
       </c>
       <c r="M315" t="n">
-        <v>1.571980555555555</v>
+        <v>1.569608496376812</v>
       </c>
     </row>
     <row r="316">
@@ -13571,37 +13571,37 @@
         <v>46067</v>
       </c>
       <c r="C316" t="n">
-        <v>0.2907767831084916</v>
+        <v>0.6658545016985661</v>
       </c>
       <c r="D316" t="n">
-        <v>3.439064114093628</v>
+        <v>1.501829600083867</v>
       </c>
       <c r="E316" t="n">
-        <v>0.3343352227193155</v>
+        <v>0.6804187058507641</v>
       </c>
       <c r="F316" t="n">
-        <v>0.7771844815968791</v>
+        <v>0.2199456323266675</v>
       </c>
       <c r="G316" t="n">
-        <v>0.4072958275444406</v>
+        <v>0.6002225325438366</v>
       </c>
       <c r="H316" t="n">
-        <v>0.6091488124714353</v>
+        <v>0.9357856977168744</v>
       </c>
       <c r="I316" t="n">
-        <v>5.142278705482186</v>
+        <v>15.26724622522133</v>
       </c>
       <c r="J316" t="n">
-        <v>0.002700810368319841</v>
+        <v>0.002673638860452837</v>
       </c>
       <c r="K316" t="n">
-        <v>0.3134280500151441</v>
+        <v>0.3174640201912212</v>
       </c>
       <c r="L316" t="n">
-        <v>0.8122535013597513</v>
+        <v>0.8271684027777777</v>
       </c>
       <c r="M316" t="n">
-        <v>1.48623670066045</v>
+        <v>1.486482743055555</v>
       </c>
     </row>
     <row r="317">
@@ -13614,37 +13614,37 @@
         <v>46068</v>
       </c>
       <c r="C317" t="n">
-        <v>0.2102616124918172</v>
+        <v>0.6321956594505016</v>
       </c>
       <c r="D317" t="n">
-        <v>4.755979886908348</v>
+        <v>1.581788778602483</v>
       </c>
       <c r="E317" t="n">
-        <v>0.3250929076542771</v>
+        <v>0.6120326357756144</v>
       </c>
       <c r="F317" t="n">
-        <v>0.6708370644005951</v>
+        <v>0.2751835627377578</v>
       </c>
       <c r="G317" t="n">
-        <v>0.3389554922238389</v>
+        <v>0.7113664332881204</v>
       </c>
       <c r="H317" t="n">
-        <v>1.827356026736117</v>
+        <v>1.098833080932041</v>
       </c>
       <c r="I317" t="n">
-        <v>3.12594660563677</v>
+        <v>14.50073944876312</v>
       </c>
       <c r="J317" t="n">
-        <v>0.001679132105142909</v>
+        <v>0.001697067961400072</v>
       </c>
       <c r="K317" t="n">
-        <v>0.3623519211877902</v>
+        <v>0.3659432362288533</v>
       </c>
       <c r="L317" t="n">
-        <v>0.8417388908059197</v>
+        <v>0.8560131944444445</v>
       </c>
       <c r="M317" t="n">
-        <v>1.14254446898244</v>
+        <v>1.152784722222222</v>
       </c>
     </row>
     <row r="318">
@@ -13657,37 +13657,37 @@
         <v>46069</v>
       </c>
       <c r="C318" t="n">
-        <v>0.3478404315435482</v>
+        <v>0.2786251516504959</v>
       </c>
       <c r="D318" t="n">
-        <v>2.874881437912442</v>
+        <v>3.589051433714025</v>
       </c>
       <c r="E318" t="n">
-        <v>0.4080193857852025</v>
+        <v>0.3723519871928017</v>
       </c>
       <c r="F318" t="n">
-        <v>0.6382499932867625</v>
+        <v>0.7120927198382135</v>
       </c>
       <c r="G318" t="n">
-        <v>0.2388872632463237</v>
+        <v>0.2329326701923812</v>
       </c>
       <c r="H318" t="n">
-        <v>0.5575287130597157</v>
+        <v>0.2448529447989121</v>
       </c>
       <c r="I318" t="n">
-        <v>6.728940548479852</v>
+        <v>6.756400137384044</v>
       </c>
       <c r="J318" t="n">
-        <v>0.004007370531132996</v>
+        <v>0.004023723885212866</v>
       </c>
       <c r="K318" t="n">
-        <v>0.2937370811267606</v>
+        <v>0.2951856290470331</v>
       </c>
       <c r="L318" t="n">
-        <v>0.8467051801830457</v>
+        <v>0.8624180555555555</v>
       </c>
       <c r="M318" t="n">
-        <v>1.403146669227263</v>
+        <v>1.395059513888889</v>
       </c>
     </row>
     <row r="319">
@@ -13700,37 +13700,37 @@
         <v>46070</v>
       </c>
       <c r="C319" t="n">
-        <v>0.2779022232236095</v>
+        <v>0.2266637379310647</v>
       </c>
       <c r="D319" t="n">
-        <v>3.598387909244491</v>
+        <v>4.411821710555794</v>
       </c>
       <c r="E319" t="n">
-        <v>0.3210443310021389</v>
+        <v>0.3070212981236177</v>
       </c>
       <c r="F319" t="n">
-        <v>1.077395231888276</v>
+        <v>1.139970741394747</v>
       </c>
       <c r="G319" t="n">
-        <v>0.120773603306114</v>
+        <v>0.1262898727648445</v>
       </c>
       <c r="H319" t="n">
-        <v>0.5584639685078406</v>
+        <v>0.2148014419488431</v>
       </c>
       <c r="I319" t="n">
-        <v>5.415096758379986</v>
+        <v>5.407286412104397</v>
       </c>
       <c r="J319" t="n">
-        <v>0.007081644575800144</v>
+        <v>0.007071430520760029</v>
       </c>
       <c r="K319" t="n">
-        <v>0.2710036357041812</v>
+        <v>0.2727882467564888</v>
       </c>
       <c r="L319" t="n">
-        <v>0.8313055134050128</v>
+        <v>0.8513187499999999</v>
       </c>
       <c r="M319" t="n">
-        <v>1.540174476344849</v>
+        <v>1.541119652777778</v>
       </c>
     </row>
     <row r="320">
@@ -13743,37 +13743,37 @@
         <v>46071</v>
       </c>
       <c r="C320" t="n">
-        <v>0.2167511020944527</v>
+        <v>0.2114976345848463</v>
       </c>
       <c r="D320" t="n">
-        <v>4.61358669154187</v>
+        <v>4.728185267711971</v>
       </c>
       <c r="E320" t="n">
-        <v>0.2738966768450472</v>
+        <v>0.2725190510112381</v>
       </c>
       <c r="F320" t="n">
-        <v>0.9309677644158552</v>
+        <v>0.9383482529326987</v>
       </c>
       <c r="G320" t="n">
-        <v>0.1486392082762455</v>
+        <v>0.1501890315297898</v>
       </c>
       <c r="H320" t="n">
-        <v>0.3144713054346175</v>
+        <v>0.3282515530570139</v>
       </c>
       <c r="I320" t="n">
-        <v>5.059029369649137</v>
+        <v>5.02330527984193</v>
       </c>
       <c r="J320" t="n">
-        <v>0.003825334733752388</v>
+        <v>0.003798322318605908</v>
       </c>
       <c r="K320" t="n">
-        <v>0.2759468469931219</v>
+        <v>0.2744220654044258</v>
       </c>
       <c r="L320" t="n">
-        <v>0.8675236369910282</v>
+        <v>0.8667044191919192</v>
       </c>
       <c r="M320" t="n">
-        <v>1.545998293493945</v>
+        <v>1.540462121212121</v>
       </c>
     </row>
     <row r="321">
@@ -13786,37 +13786,37 @@
         <v>46072</v>
       </c>
       <c r="C321" t="n">
-        <v>0.3760325292300464</v>
+        <v>0.3142992234644668</v>
       </c>
       <c r="D321" t="n">
-        <v>2.659344397804019</v>
+        <v>3.18168142121756</v>
       </c>
       <c r="E321" t="n">
-        <v>0.4779129651883251</v>
+        <v>0.4367828796638205</v>
       </c>
       <c r="F321" t="n">
-        <v>0.6418596038394272</v>
+        <v>0.7550626413946721</v>
       </c>
       <c r="G321" t="n">
-        <v>0.112880085782671</v>
+        <v>0.1235095490661863</v>
       </c>
       <c r="H321" t="n">
-        <v>0.360466590910762</v>
+        <v>0.1587331241534058</v>
       </c>
       <c r="I321" t="n">
-        <v>7.528716156172969</v>
+        <v>7.520002184166466</v>
       </c>
       <c r="J321" t="n">
-        <v>0.004280529918026246</v>
+        <v>0.004275575498560173</v>
       </c>
       <c r="K321" t="n">
-        <v>0.330179921492625</v>
+        <v>0.3330382215201328</v>
       </c>
       <c r="L321" t="n">
-        <v>0.8621247129819499</v>
+        <v>0.8726638888888889</v>
       </c>
       <c r="M321" t="n">
-        <v>1.414130751215159</v>
+        <v>1.410946527777778</v>
       </c>
     </row>
     <row r="322">
@@ -13829,37 +13829,37 @@
         <v>46073</v>
       </c>
       <c r="C322" t="n">
-        <v>0.2445020568663155</v>
+        <v>0.2386386866272707</v>
       </c>
       <c r="D322" t="n">
-        <v>4.089945143270358</v>
+        <v>4.190435398942243</v>
       </c>
       <c r="E322" t="n">
-        <v>0.3336200037835133</v>
+        <v>0.3294306698585029</v>
       </c>
       <c r="F322" t="n">
-        <v>0.8895705346933372</v>
+        <v>0.9094480652549295</v>
       </c>
       <c r="G322" t="n">
-        <v>0.07942270570256574</v>
+        <v>0.08043271559496219</v>
       </c>
       <c r="H322" t="n">
-        <v>0.1986276670475679</v>
+        <v>0.1731918894780276</v>
       </c>
       <c r="I322" t="n">
-        <v>5.59114711560786</v>
+        <v>5.603758826520487</v>
       </c>
       <c r="J322" t="n">
-        <v>0.006468849782400072</v>
+        <v>0.006483441289599928</v>
       </c>
       <c r="K322" t="n">
-        <v>0.2621996676284666</v>
+        <v>0.2632047917738793</v>
       </c>
       <c r="L322" t="n">
-        <v>0.867631798245614</v>
+        <v>0.8695097222222222</v>
       </c>
       <c r="M322" t="n">
-        <v>1.498311458333333</v>
+        <v>1.495883333333333</v>
       </c>
     </row>
     <row r="323">
@@ -13872,37 +13872,37 @@
         <v>46074</v>
       </c>
       <c r="C323" t="n">
-        <v>0.5644737118680579</v>
+        <v>0.6517519591861886</v>
       </c>
       <c r="D323" t="n">
-        <v>1.771561684760518</v>
+        <v>1.53432603601016</v>
       </c>
       <c r="E323" t="n">
-        <v>0.5759850812685037</v>
+        <v>0.7653493334564807</v>
       </c>
       <c r="F323" t="n">
-        <v>0.2634911218255498</v>
+        <v>0.1570236759554615</v>
       </c>
       <c r="G323" t="n">
-        <v>0.8170455727249658</v>
+        <v>0.6893056361983576</v>
       </c>
       <c r="H323" t="n">
-        <v>0.9425415898734815</v>
+        <v>0.97159346258621</v>
       </c>
       <c r="I323" t="n">
-        <v>11.18873995879386</v>
+        <v>14.73130160544578</v>
       </c>
       <c r="J323" t="n">
-        <v>0.001705117809454611</v>
+        <v>0.001700921192967293</v>
       </c>
       <c r="K323" t="n">
-        <v>0.3155466862125447</v>
+        <v>0.3168525581094946</v>
       </c>
       <c r="L323" t="n">
-        <v>0.8565559070314267</v>
+        <v>0.8595840277777778</v>
       </c>
       <c r="M323" t="n">
-        <v>1.257690909022714</v>
+        <v>1.257376458333333</v>
       </c>
     </row>
     <row r="324">
@@ -13915,37 +13915,37 @@
         <v>46075</v>
       </c>
       <c r="C324" t="n">
-        <v>0.2275116672733582</v>
+        <v>0.6363653974030454</v>
       </c>
       <c r="D324" t="n">
-        <v>4.395378979832656</v>
+        <v>1.571424222751453</v>
       </c>
       <c r="E324" t="n">
-        <v>0.7481007493546525</v>
+        <v>0.7370350116538432</v>
       </c>
       <c r="F324" t="n">
-        <v>0.2775633334118789</v>
+        <v>0.2651366186141378</v>
       </c>
       <c r="G324" t="n">
-        <v>0.5024680763476866</v>
+        <v>0.5100120598057006</v>
       </c>
       <c r="H324" t="n">
-        <v>3.196547416574722</v>
+        <v>1.110986290531485</v>
       </c>
       <c r="I324" t="n">
-        <v>3.81791040653629</v>
+        <v>14.55605098199664</v>
       </c>
       <c r="J324" t="n">
-        <v>0.001404913038095152</v>
+        <v>0.001409927667520058</v>
       </c>
       <c r="K324" t="n">
-        <v>0.09226271065961927</v>
+        <v>0.09806685311753938</v>
       </c>
       <c r="L324" t="n">
-        <v>0.8586095238095239</v>
+        <v>0.8622493055555557</v>
       </c>
       <c r="M324" t="n">
-        <v>2.48886768907563</v>
+        <v>2.375972569444444</v>
       </c>
     </row>
     <row r="325">
@@ -13958,37 +13958,37 @@
         <v>46076</v>
       </c>
       <c r="C325" t="n">
-        <v>0.2554075985761329</v>
+        <v>0.2393533091123313</v>
       </c>
       <c r="D325" t="n">
-        <v>3.915310294505259</v>
+        <v>4.17792427315341</v>
       </c>
       <c r="E325" t="n">
-        <v>0.3394207019403488</v>
+        <v>0.3309414696219769</v>
       </c>
       <c r="F325" t="n">
-        <v>1.095279956873408</v>
+        <v>1.134126046595017</v>
       </c>
       <c r="G325" t="n">
-        <v>0.1314175903250847</v>
+        <v>0.1347847122525961</v>
       </c>
       <c r="H325" t="n">
-        <v>0.186722989101861</v>
+        <v>0.1697490137975424</v>
       </c>
       <c r="I325" t="n">
-        <v>5.759913454316966</v>
+        <v>5.840590092979689</v>
       </c>
       <c r="J325" t="n">
-        <v>0.003982759230244311</v>
+        <v>0.0040385440315</v>
       </c>
       <c r="K325" t="n">
-        <v>0.2775525721797517</v>
+        <v>0.2771810987977096</v>
       </c>
       <c r="L325" t="n">
-        <v>0.8570279365432374</v>
+        <v>0.859</v>
       </c>
       <c r="M325" t="n">
-        <v>1.456062277284041</v>
+        <v>1.441812777777778</v>
       </c>
     </row>
     <row r="326">
@@ -14001,37 +14001,37 @@
         <v>46077</v>
       </c>
       <c r="C326" t="n">
-        <v>0.2493769027545836</v>
+        <v>0.214402618928611</v>
       </c>
       <c r="D326" t="n">
-        <v>4.009994466023657</v>
+        <v>4.664122131516347</v>
       </c>
       <c r="E326" t="n">
-        <v>0.3111133709932039</v>
+        <v>0.300685288392818</v>
       </c>
       <c r="F326" t="n">
-        <v>0.8279339728021268</v>
+        <v>0.8557133623857159</v>
       </c>
       <c r="G326" t="n">
-        <v>0.1001087466298913</v>
+        <v>0.1035806234365603</v>
       </c>
       <c r="H326" t="n">
-        <v>0.3479920358498124</v>
+        <v>0.1391397637836548</v>
       </c>
       <c r="I326" t="n">
-        <v>5.065587342018174</v>
+        <v>5.045681232109857</v>
       </c>
       <c r="J326" t="n">
-        <v>0.00499400155</v>
+        <v>0.004974376748960246</v>
       </c>
       <c r="K326" t="n">
-        <v>0.309747094433826</v>
+        <v>0.3133153898590534</v>
       </c>
       <c r="L326" t="n">
-        <v>0.838076697177727</v>
+        <v>0.8478208333333334</v>
       </c>
       <c r="M326" t="n">
-        <v>1.542971166098353</v>
+        <v>1.522618125</v>
       </c>
     </row>
     <row r="327">
@@ -14044,37 +14044,37 @@
         <v>46078</v>
       </c>
       <c r="C327" t="n">
-        <v>0.2473390033509216</v>
+        <v>0.2064594991000644</v>
       </c>
       <c r="D327" t="n">
-        <v>4.04303399970126</v>
+        <v>4.843564981794959</v>
       </c>
       <c r="E327" t="n">
-        <v>0.3119953325693995</v>
+        <v>0.2918152227878672</v>
       </c>
       <c r="F327" t="n">
-        <v>1.061206253512426</v>
+        <v>1.115386505721498</v>
       </c>
       <c r="G327" t="n">
-        <v>0.09000683797822745</v>
+        <v>0.09623114613506957</v>
       </c>
       <c r="H327" t="n">
-        <v>0.1296133167081826</v>
+        <v>0.1225023539996944</v>
       </c>
       <c r="I327" t="n">
-        <v>4.996005388431217</v>
+        <v>4.98999589480868</v>
       </c>
       <c r="J327" t="n">
-        <v>0.00544856545368719</v>
+        <v>0.005442011593793097</v>
       </c>
       <c r="K327" t="n">
-        <v>0.2902330780764976</v>
+        <v>0.2897588594265528</v>
       </c>
       <c r="L327" t="n">
-        <v>0.8472869648869649</v>
+        <v>0.85380625</v>
       </c>
       <c r="M327" t="n">
-        <v>1.546826186353329</v>
+        <v>1.539671527777778</v>
       </c>
     </row>
     <row r="328">
@@ -14087,37 +14087,37 @@
         <v>46079</v>
       </c>
       <c r="C328" t="n">
-        <v>0.3573188931413683</v>
+        <v>0.2815830501845067</v>
       </c>
       <c r="D328" t="n">
-        <v>2.79862055769988</v>
+        <v>3.551350123328632</v>
       </c>
       <c r="E328" t="n">
-        <v>0.3989213629606124</v>
+        <v>0.3684431880214059</v>
       </c>
       <c r="F328" t="n">
-        <v>0.6230086530143061</v>
+        <v>0.7059885751760491</v>
       </c>
       <c r="G328" t="n">
-        <v>0.1462369303342058</v>
+        <v>0.158333869265913</v>
       </c>
       <c r="H328" t="n">
-        <v>0.672833187527888</v>
+        <v>0.2927527988506103</v>
       </c>
       <c r="I328" t="n">
-        <v>6.462206939648571</v>
+        <v>6.586299679576427</v>
       </c>
       <c r="J328" t="n">
-        <v>0.003513179221490955</v>
+        <v>0.003521434534173112</v>
       </c>
       <c r="K328" t="n">
-        <v>0.3034780961758167</v>
+        <v>0.3053194834414337</v>
       </c>
       <c r="L328" t="n">
-        <v>0.849682703918888</v>
+        <v>0.8613395833333333</v>
       </c>
       <c r="M328" t="n">
-        <v>1.449149957279563</v>
+        <v>1.425945625</v>
       </c>
     </row>
     <row r="329">
@@ -14130,22 +14130,22 @@
         <v>46080</v>
       </c>
       <c r="C329" t="n">
-        <v>0.2615570568864216</v>
+        <v>0.2556961689072306</v>
       </c>
       <c r="D329" t="n">
-        <v>3.823257578686701</v>
+        <v>3.910891603396729</v>
       </c>
       <c r="E329" t="n">
-        <v>0.3558607903298955</v>
+        <v>0.3475650060150218</v>
       </c>
       <c r="F329" t="n">
-        <v>0.7655688316892528</v>
+        <v>0.8001403509347118</v>
       </c>
       <c r="G329" t="n">
-        <v>0.1965622793679224</v>
+        <v>0.2012538859619584</v>
       </c>
       <c r="H329" t="n">
-        <v>0.204994739464966</v>
+        <v>0.2070360751120563</v>
       </c>
       <c r="I329" t="n">
         <v>6.131544869633232</v>
@@ -14154,13 +14154,13 @@
         <v>0.00629778870317804</v>
       </c>
       <c r="K329" t="n">
-        <v>0.2707176543610253</v>
+        <v>0.2708391036978406</v>
       </c>
       <c r="L329" t="n">
-        <v>0.8536505892255892</v>
+        <v>0.8546015151515153</v>
       </c>
       <c r="M329" t="n">
-        <v>1.443423282828283</v>
+        <v>1.443978838383838</v>
       </c>
     </row>
     <row r="330">
@@ -14173,37 +14173,37 @@
         <v>46081</v>
       </c>
       <c r="C330" t="n">
-        <v>0.661852709172418</v>
+        <v>0.6699139047914663</v>
       </c>
       <c r="D330" t="n">
-        <v>1.510910186120417</v>
+        <v>1.492729129590592</v>
       </c>
       <c r="E330" t="n">
-        <v>0.6943113181140568</v>
+        <v>0.701125145592249</v>
       </c>
       <c r="F330" t="n">
-        <v>0.3562405977818858</v>
+        <v>0.269148800103335</v>
       </c>
       <c r="G330" t="n">
-        <v>0.3168806062712582</v>
+        <v>0.531357508677041</v>
       </c>
       <c r="H330" t="n">
-        <v>0.8036526929660559</v>
+        <v>0.8664521975983976</v>
       </c>
       <c r="I330" t="n">
-        <v>16.53381589523741</v>
+        <v>16.48616440920722</v>
       </c>
       <c r="J330" t="n">
-        <v>0.002306810845714183</v>
+        <v>0.002300162473342955</v>
       </c>
       <c r="K330" t="n">
-        <v>0.3103521286261414</v>
+        <v>0.3139094941193616</v>
       </c>
       <c r="L330" t="n">
-        <v>0.8565873542170492</v>
+        <v>0.8553360809178744</v>
       </c>
       <c r="M330" t="n">
-        <v>1.361392336383829</v>
+        <v>1.341075600845411</v>
       </c>
     </row>
     <row r="331">
@@ -14216,37 +14216,37 @@
         <v>46082</v>
       </c>
       <c r="C331" t="n">
-        <v>0.2461733724352257</v>
+        <v>0.6946498459753002</v>
       </c>
       <c r="D331" t="n">
-        <v>4.062177765644108</v>
+        <v>1.439574205326402</v>
       </c>
       <c r="E331" t="n">
-        <v>0.2343089450121791</v>
+        <v>0.7026572108428287</v>
       </c>
       <c r="F331" t="n">
-        <v>0.9152273910835963</v>
+        <v>0.2870078880171892</v>
       </c>
       <c r="G331" t="n">
-        <v>0.3795117377262617</v>
+        <v>0.5231389851337762</v>
       </c>
       <c r="H331" t="n">
-        <v>1.151907483802164</v>
+        <v>0.9658124982823834</v>
       </c>
       <c r="I331" t="n">
-        <v>3.833465503567782</v>
+        <v>15.94310906131277</v>
       </c>
       <c r="J331" t="n">
-        <v>0.002266760891332851</v>
+        <v>0.002280555557359957</v>
       </c>
       <c r="K331" t="n">
-        <v>0.3537970522951244</v>
+        <v>0.3552904551829874</v>
       </c>
       <c r="L331" t="n">
-        <v>0.8388954208437761</v>
+        <v>0.8525361111111112</v>
       </c>
       <c r="M331" t="n">
-        <v>1.09267709727042</v>
+        <v>1.091589807692308</v>
       </c>
     </row>
     <row r="332">
@@ -14259,37 +14259,37 @@
         <v>46083</v>
       </c>
       <c r="C332" t="n">
-        <v>0.2181223797223631</v>
+        <v>0.2047006610636065</v>
       </c>
       <c r="D332" t="n">
-        <v>4.584582293998668</v>
+        <v>4.885182074176451</v>
       </c>
       <c r="E332" t="n">
-        <v>0.2913251201228754</v>
+        <v>0.2880839574344897</v>
       </c>
       <c r="F332" t="n">
-        <v>1.058545439196658</v>
+        <v>1.079470954407087</v>
       </c>
       <c r="G332" t="n">
-        <v>0.1054117050441238</v>
+        <v>0.1065976665546179</v>
       </c>
       <c r="H332" t="n">
-        <v>0.1743819077944617</v>
+        <v>0.1316771286386765</v>
       </c>
       <c r="I332" t="n">
-        <v>4.882063764775336</v>
+        <v>4.879930047799014</v>
       </c>
       <c r="J332" t="n">
-        <v>0.01139775523956913</v>
+        <v>0.01139277382494236</v>
       </c>
       <c r="K332" t="n">
-        <v>0.3118350281575002</v>
+        <v>0.3131762663389314</v>
       </c>
       <c r="L332" t="n">
-        <v>0.866137806489562</v>
+        <v>0.8695152390214158</v>
       </c>
       <c r="M332" t="n">
-        <v>1.294800339139747</v>
+        <v>1.270909968219313</v>
       </c>
     </row>
     <row r="333">
@@ -14302,37 +14302,37 @@
         <v>46084</v>
       </c>
       <c r="C333" t="n">
-        <v>0.2293711326615225</v>
+        <v>0.2121456151339614</v>
       </c>
       <c r="D333" t="n">
-        <v>4.359746531293789</v>
+        <v>4.713743432163517</v>
       </c>
       <c r="E333" t="n">
-        <v>0.3187635393095411</v>
+        <v>0.295902487758366</v>
       </c>
       <c r="F333" t="n">
-        <v>0.7762118240977036</v>
+        <v>0.8486612040361026</v>
       </c>
       <c r="G333" t="n">
-        <v>0.04486141739409488</v>
+        <v>0.1031441533059334</v>
       </c>
       <c r="H333" t="n">
-        <v>0.1586954376120232</v>
+        <v>0.1508330336228831</v>
       </c>
       <c r="I333" t="n">
-        <v>5.036794232469142</v>
+        <v>5.051364883849607</v>
       </c>
       <c r="J333" t="n">
-        <v>0.01092408046139513</v>
+        <v>0.01095568210337388</v>
       </c>
       <c r="K333" t="n">
-        <v>0.3221536940382374</v>
+        <v>0.3249190300678226</v>
       </c>
       <c r="L333" t="n">
-        <v>0.8381350530160766</v>
+        <v>0.840854731181557</v>
       </c>
       <c r="M333" t="n">
-        <v>1.607554860385983</v>
+        <v>1.606863995350759</v>
       </c>
     </row>
     <row r="334">
@@ -14345,37 +14345,37 @@
         <v>46085</v>
       </c>
       <c r="C334" t="n">
-        <v>0.2896251016259764</v>
+        <v>0.2688764519440303</v>
       </c>
       <c r="D334" t="n">
-        <v>3.452739401336166</v>
+        <v>3.719180288083248</v>
       </c>
       <c r="E334" t="n">
-        <v>0.3606056526201806</v>
+        <v>0.3555779848054487</v>
       </c>
       <c r="F334" t="n">
-        <v>0.7039189868451009</v>
+        <v>0.7478658395946826</v>
       </c>
       <c r="G334" t="n">
-        <v>0.2405832759138892</v>
+        <v>0.2259171693058295</v>
       </c>
       <c r="H334" t="n">
-        <v>0.4094888656476496</v>
+        <v>0.2685019610351606</v>
       </c>
       <c r="I334" t="n">
-        <v>6.348266256170776</v>
+        <v>6.359945147593077</v>
       </c>
       <c r="J334" t="n">
-        <v>0.007384240175872649</v>
+        <v>0.007397824946228868</v>
       </c>
       <c r="K334" t="n">
-        <v>0.2965271704596892</v>
+        <v>0.296310503027635</v>
       </c>
       <c r="L334" t="n">
-        <v>0.8311930431162854</v>
+        <v>0.8393931983044579</v>
       </c>
       <c r="M334" t="n">
-        <v>1.686020573869447</v>
+        <v>1.686615839329826</v>
       </c>
     </row>
     <row r="335">
@@ -14388,37 +14388,37 @@
         <v>46086</v>
       </c>
       <c r="C335" t="n">
-        <v>0.3613130589189197</v>
+        <v>0.3486939694431138</v>
       </c>
       <c r="D335" t="n">
-        <v>2.767682969976473</v>
+        <v>2.867844263544514</v>
       </c>
       <c r="E335" t="n">
-        <v>0.4714133133424473</v>
+        <v>0.4663909013888259</v>
       </c>
       <c r="F335" t="n">
-        <v>0.688716515356453</v>
+        <v>0.7047489468402954</v>
       </c>
       <c r="G335" t="n">
-        <v>0.1465075560948265</v>
+        <v>0.2463327019217022</v>
       </c>
       <c r="H335" t="n">
-        <v>0.2993393399760784</v>
+        <v>0.2429294937236192</v>
       </c>
       <c r="I335" t="n">
-        <v>8.21996712702331</v>
+        <v>8.254282411551488</v>
       </c>
       <c r="J335" t="n">
-        <v>0.006479896948611447</v>
+        <v>0.006506948091769168</v>
       </c>
       <c r="K335" t="n">
-        <v>0.3135309054295451</v>
+        <v>0.3136567525784734</v>
       </c>
       <c r="L335" t="n">
-        <v>0.8570704576343958</v>
+        <v>0.8602951203726863</v>
       </c>
       <c r="M335" t="n">
-        <v>1.90115464127556</v>
+        <v>1.899221479003886</v>
       </c>
     </row>
     <row r="336">
@@ -14431,37 +14431,37 @@
         <v>46087</v>
       </c>
       <c r="C336" t="n">
-        <v>0.4193274396298945</v>
+        <v>0.3485501692314891</v>
       </c>
       <c r="D336" t="n">
-        <v>2.38477119666344</v>
+        <v>2.869027440740823</v>
       </c>
       <c r="E336" t="n">
-        <v>0.4876278704093439</v>
+        <v>0.4268893281551918</v>
       </c>
       <c r="F336" t="n">
-        <v>0.4890077120773541</v>
+        <v>0.5568750773010762</v>
       </c>
       <c r="G336" t="n">
-        <v>0.2522631799303597</v>
+        <v>0.2881556157510948</v>
       </c>
       <c r="H336" t="n">
-        <v>0.5797998745101635</v>
+        <v>0.449465092541106</v>
       </c>
       <c r="I336" t="n">
-        <v>8.201399743119373</v>
+        <v>8.12739607412445</v>
       </c>
       <c r="J336" t="n">
-        <v>0.004339567582156444</v>
+        <v>0.004300410373266532</v>
       </c>
       <c r="K336" t="n">
-        <v>0.3287842708845661</v>
+        <v>0.3311915763142386</v>
       </c>
       <c r="L336" t="n">
-        <v>0.851048549440197</v>
+        <v>0.8625732621606526</v>
       </c>
       <c r="M336" t="n">
-        <v>1.793445101692906</v>
+        <v>1.795258730498108</v>
       </c>
     </row>
     <row r="337">
@@ -14474,37 +14474,37 @@
         <v>46088</v>
       </c>
       <c r="C337" t="n">
-        <v>0.6051453921724883</v>
+        <v>0.573815093307026</v>
       </c>
       <c r="D337" t="n">
-        <v>1.65249543817887</v>
+        <v>1.742721674044463</v>
       </c>
       <c r="E337" t="n">
-        <v>0.6414074612187748</v>
+        <v>0.6205947326329517</v>
       </c>
       <c r="F337" t="n">
-        <v>0.2599122209853285</v>
+        <v>0.2376772354761874</v>
       </c>
       <c r="G337" t="n">
-        <v>0.6479182438303287</v>
+        <v>0.6696473141004422</v>
       </c>
       <c r="H337" t="n">
-        <v>0.7625523568045063</v>
+        <v>0.7738638267483</v>
       </c>
       <c r="I337" t="n">
-        <v>13.62217638464642</v>
+        <v>13.4034445955629</v>
       </c>
       <c r="J337" t="n">
-        <v>0.003167768619948327</v>
+        <v>0.003116903642276706</v>
       </c>
       <c r="K337" t="n">
-        <v>0.3143149214114223</v>
+        <v>0.3143940727103471</v>
       </c>
       <c r="L337" t="n">
-        <v>0.8358625558590751</v>
+        <v>0.8374671260672842</v>
       </c>
       <c r="M337" t="n">
-        <v>1.515695617515302</v>
+        <v>1.489160289613727</v>
       </c>
     </row>
     <row r="338">
@@ -14517,37 +14517,37 @@
         <v>46089</v>
       </c>
       <c r="C338" t="n">
-        <v>0.2213651787049339</v>
+        <v>0.6761888378297394</v>
       </c>
       <c r="D338" t="n">
-        <v>4.517422323828709</v>
+        <v>1.47887682264846</v>
       </c>
       <c r="E338" t="n">
-        <v>0.2066456025316323</v>
+        <v>0.8435295416976366</v>
       </c>
       <c r="F338" t="n">
-        <v>1.03882154946239</v>
+        <v>0.1957650448652403</v>
       </c>
       <c r="G338" t="n">
-        <v>0.2722967955830185</v>
+        <v>0.7074809202696661</v>
       </c>
       <c r="H338" t="n">
-        <v>1.213693047318271</v>
+        <v>1.233530671618116</v>
       </c>
       <c r="I338" t="n">
-        <v>3.900091266187371</v>
+        <v>15.60760545394997</v>
       </c>
       <c r="J338" t="n">
-        <v>0.002148133567997152</v>
+        <v>0.002143178610589619</v>
       </c>
       <c r="K338" t="n">
-        <v>0.3558147997530159</v>
+        <v>0.3575976079725227</v>
       </c>
       <c r="L338" t="n">
-        <v>0.840371486671792</v>
+        <v>0.850091019182134</v>
       </c>
       <c r="M338" t="n">
-        <v>1.339595569203737</v>
+        <v>1.339795734878083</v>
       </c>
     </row>
     <row r="339">
@@ -14560,37 +14560,37 @@
         <v>46090</v>
       </c>
       <c r="C339" t="n">
-        <v>0.3837890883652313</v>
+        <v>0.369284988638939</v>
       </c>
       <c r="D339" t="n">
-        <v>2.605597788773906</v>
+        <v>2.707935688601006</v>
       </c>
       <c r="E339" t="n">
-        <v>0.4900161450673422</v>
+        <v>0.4804330319936984</v>
       </c>
       <c r="F339" t="n">
-        <v>0.4984426845704988</v>
+        <v>0.502637733815869</v>
       </c>
       <c r="G339" t="n">
-        <v>0.1388244731932012</v>
+        <v>0.1415935805097375</v>
       </c>
       <c r="H339" t="n">
-        <v>0.3496516934915755</v>
+        <v>0.3059508654503765</v>
       </c>
       <c r="I339" t="n">
-        <v>8.560827684752271</v>
+        <v>8.62365659043083</v>
       </c>
       <c r="J339" t="n">
-        <v>0.003870448321159658</v>
+        <v>0.003898853989566814</v>
       </c>
       <c r="K339" t="n">
-        <v>0.3079690149762999</v>
+        <v>0.3090096936350965</v>
       </c>
       <c r="L339" t="n">
-        <v>0.8448908192817332</v>
+        <v>0.8459893985342749</v>
       </c>
       <c r="M339" t="n">
-        <v>1.67799400293386</v>
+        <v>1.674028385794495</v>
       </c>
     </row>
     <row r="340">
@@ -14603,37 +14603,37 @@
         <v>46091</v>
       </c>
       <c r="C340" t="n">
-        <v>0.2322412876272421</v>
+        <v>0.2125275572702686</v>
       </c>
       <c r="D340" t="n">
-        <v>4.305866584778181</v>
+        <v>4.705272167262116</v>
       </c>
       <c r="E340" t="n">
-        <v>0.3098367060634977</v>
+        <v>0.2997268910326205</v>
       </c>
       <c r="F340" t="n">
-        <v>0.9396872797231078</v>
+        <v>0.9849047011845592</v>
       </c>
       <c r="G340" t="n">
-        <v>0.1119420655733522</v>
+        <v>0.1157178815277429</v>
       </c>
       <c r="H340" t="n">
-        <v>0.1771266287289659</v>
+        <v>0.1272121083770725</v>
       </c>
       <c r="I340" t="n">
-        <v>5.073931368306589</v>
+        <v>5.073042903154941</v>
       </c>
       <c r="J340" t="n">
-        <v>0.01010003952895152</v>
+        <v>0.01009827097267822</v>
       </c>
       <c r="K340" t="n">
-        <v>0.3030582268821165</v>
+        <v>0.3059579553480526</v>
       </c>
       <c r="L340" t="n">
-        <v>0.8360425489139203</v>
+        <v>0.8440163702699303</v>
       </c>
       <c r="M340" t="n">
-        <v>1.831781699588833</v>
+        <v>1.824209509243235</v>
       </c>
     </row>
     <row r="341">
@@ -14646,37 +14646,37 @@
         <v>46092</v>
       </c>
       <c r="C341" t="n">
-        <v>0.4120000912330334</v>
+        <v>0.3446617955302063</v>
       </c>
       <c r="D341" t="n">
-        <v>2.427183928545261</v>
+        <v>2.90139497028286</v>
       </c>
       <c r="E341" t="n">
-        <v>0.4486880672281404</v>
+        <v>0.4447764318000895</v>
       </c>
       <c r="F341" t="n">
-        <v>0.5679418556019838</v>
+        <v>0.5791594242038587</v>
       </c>
       <c r="G341" t="n">
-        <v>0.2200603141125843</v>
+        <v>0.2219956588373643</v>
       </c>
       <c r="H341" t="n">
-        <v>0.7001868592588935</v>
+        <v>0.3247306121996968</v>
       </c>
       <c r="I341" t="n">
-        <v>8.133970601705197</v>
+        <v>8.072862734072755</v>
       </c>
       <c r="J341" t="n">
-        <v>0.005456461133016709</v>
+        <v>0.005415468520554101</v>
       </c>
       <c r="K341" t="n">
-        <v>0.3012936339387081</v>
+        <v>0.3040752369243107</v>
       </c>
       <c r="L341" t="n">
-        <v>0.8490017885378254</v>
+        <v>0.8603520885164236</v>
       </c>
       <c r="M341" t="n">
-        <v>1.816711929291791</v>
+        <v>1.79589385759953</v>
       </c>
     </row>
     <row r="342">
@@ -14689,37 +14689,37 @@
         <v>46093</v>
       </c>
       <c r="C342" t="n">
-        <v>0.5594587261627938</v>
+        <v>0.4718581913986053</v>
       </c>
       <c r="D342" t="n">
-        <v>1.787441956368762</v>
+        <v>2.119280788653817</v>
       </c>
       <c r="E342" t="n">
-        <v>0.668242362061276</v>
+        <v>0.6647141396259132</v>
       </c>
       <c r="F342" t="n">
-        <v>0.5141821174641984</v>
+        <v>0.5197411704567795</v>
       </c>
       <c r="G342" t="n">
-        <v>0.1271210660539748</v>
+        <v>0.1277958093316059</v>
       </c>
       <c r="H342" t="n">
-        <v>0.3488372358619973</v>
+        <v>0.1295990107754753</v>
       </c>
       <c r="I342" t="n">
-        <v>8.213223719491705</v>
+        <v>8.174187391205118</v>
       </c>
       <c r="J342" t="n">
-        <v>0.01224779319227569</v>
+        <v>0.0121895811074514</v>
       </c>
       <c r="K342" t="n">
-        <v>0.2879695181703519</v>
+        <v>0.2942361731284392</v>
       </c>
       <c r="L342" t="n">
-        <v>0.8092853300840299</v>
+        <v>0.8367364223607462</v>
       </c>
       <c r="M342" t="n">
-        <v>1.802810498987791</v>
+        <v>1.774414178468899</v>
       </c>
     </row>
     <row r="343">
@@ -20052,6 +20052,1339 @@
       </c>
       <c r="M466" t="n">
         <v>2.18782387039742</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C467" t="n">
+        <v>0.2940412501409206</v>
+      </c>
+      <c r="D467" t="n">
+        <v>3.400883377827925</v>
+      </c>
+      <c r="E467" t="n">
+        <v>0.4058212373422499</v>
+      </c>
+      <c r="F467" t="n">
+        <v>0.8995738429309595</v>
+      </c>
+      <c r="G467" t="n">
+        <v>0.1439956800547604</v>
+      </c>
+      <c r="H467" t="n">
+        <v>0.173675671090672</v>
+      </c>
+      <c r="I467" t="n">
+        <v>7.012550682833611</v>
+      </c>
+      <c r="J467" t="n">
+        <v>0.002800152919600108</v>
+      </c>
+      <c r="K467" t="n">
+        <v>11.10967308489649</v>
+      </c>
+      <c r="L467" t="n">
+        <v>0.8227444444444444</v>
+      </c>
+      <c r="M467" t="n">
+        <v>13.50135902777778</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="C468" t="n">
+        <v>0.3929708461834536</v>
+      </c>
+      <c r="D468" t="n">
+        <v>2.544718036241198</v>
+      </c>
+      <c r="E468" t="n">
+        <v>0.5168362265973706</v>
+      </c>
+      <c r="F468" t="n">
+        <v>0.5809595938523491</v>
+      </c>
+      <c r="G468" t="n">
+        <v>0.2167896583689557</v>
+      </c>
+      <c r="H468" t="n">
+        <v>0.2810176181182544</v>
+      </c>
+      <c r="I468" t="n">
+        <v>9.272861929279893</v>
+      </c>
+      <c r="J468" t="n">
+        <v>0.001901035694059993</v>
+      </c>
+      <c r="K468" t="n">
+        <v>11.26926880121813</v>
+      </c>
+      <c r="L468" t="n">
+        <v>0.8686930555555555</v>
+      </c>
+      <c r="M468" t="n">
+        <v>13.7708546207265</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B469" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="C469" t="n">
+        <v>0.2886930083476249</v>
+      </c>
+      <c r="D469" t="n">
+        <v>3.46388714338335</v>
+      </c>
+      <c r="E469" t="n">
+        <v>0.3766644832786595</v>
+      </c>
+      <c r="F469" t="n">
+        <v>0.7883631512282951</v>
+      </c>
+      <c r="G469" t="n">
+        <v>0.2691679860506004</v>
+      </c>
+      <c r="H469" t="n">
+        <v>0.29933817360248</v>
+      </c>
+      <c r="I469" t="n">
+        <v>6.819183029527917</v>
+      </c>
+      <c r="J469" t="n">
+        <v>0.001515796296266534</v>
+      </c>
+      <c r="K469" t="n">
+        <v>11.36542178552468</v>
+      </c>
+      <c r="L469" t="n">
+        <v>0.8382215277777778</v>
+      </c>
+      <c r="M469" t="n">
+        <v>13.81769513888889</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="n">
+        <v>46066</v>
+      </c>
+      <c r="C470" t="n">
+        <v>0.2397270748905629</v>
+      </c>
+      <c r="D470" t="n">
+        <v>4.171410344269653</v>
+      </c>
+      <c r="E470" t="n">
+        <v>0.3226422812109022</v>
+      </c>
+      <c r="F470" t="n">
+        <v>1.070692675592261</v>
+      </c>
+      <c r="G470" t="n">
+        <v>0.1785371718731205</v>
+      </c>
+      <c r="H470" t="n">
+        <v>0.2290358906853256</v>
+      </c>
+      <c r="I470" t="n">
+        <v>5.686711116038337</v>
+      </c>
+      <c r="J470" t="n">
+        <v>0.002090210122080051</v>
+      </c>
+      <c r="K470" t="n">
+        <v>11.20209759994862</v>
+      </c>
+      <c r="L470" t="n">
+        <v>0.8244631944444444</v>
+      </c>
+      <c r="M470" t="n">
+        <v>13.62218590277778</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B471" s="2" t="n">
+        <v>46067</v>
+      </c>
+      <c r="C471" t="n">
+        <v>0.6797481299229999</v>
+      </c>
+      <c r="D471" t="n">
+        <v>1.471133138848469</v>
+      </c>
+      <c r="E471" t="n">
+        <v>0.71912656450061</v>
+      </c>
+      <c r="F471" t="n">
+        <v>0.187408598410842</v>
+      </c>
+      <c r="G471" t="n">
+        <v>0.8062696067190724</v>
+      </c>
+      <c r="H471" t="n">
+        <v>0.8357239051308468</v>
+      </c>
+      <c r="I471" t="n">
+        <v>15.71862380768329</v>
+      </c>
+      <c r="J471" t="n">
+        <v>0.0005367596847433141</v>
+      </c>
+      <c r="K471" t="n">
+        <v>11.45575686466419</v>
+      </c>
+      <c r="L471" t="n">
+        <v>0.750207638888889</v>
+      </c>
+      <c r="M471" t="n">
+        <v>13.77276121527778</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="n">
+        <v>46068</v>
+      </c>
+      <c r="C472" t="n">
+        <v>0.9944026296245921</v>
+      </c>
+      <c r="D472" t="n">
+        <v>1.005628877286378</v>
+      </c>
+      <c r="E472" t="n">
+        <v>0.9949759473708072</v>
+      </c>
+      <c r="F472" t="n">
+        <v>0.002737513290029896</v>
+      </c>
+      <c r="G472" t="n">
+        <v>0.9963399171970596</v>
+      </c>
+      <c r="H472" t="n">
+        <v>0.9982713619930313</v>
+      </c>
+      <c r="I472" t="n">
+        <v>22.87270645916169</v>
+      </c>
+      <c r="J472" t="n">
+        <v>0.0004568343159834659</v>
+      </c>
+      <c r="K472" t="n">
+        <v>11.43047127174193</v>
+      </c>
+      <c r="L472" t="n">
+        <v>0.7192423611111111</v>
+      </c>
+      <c r="M472" t="n">
+        <v>13.57859402777778</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B473" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="C473" t="n">
+        <v>0.4351470040807153</v>
+      </c>
+      <c r="D473" t="n">
+        <v>2.298073962643002</v>
+      </c>
+      <c r="E473" t="n">
+        <v>0.5214792636802292</v>
+      </c>
+      <c r="F473" t="n">
+        <v>0.4358417521741886</v>
+      </c>
+      <c r="G473" t="n">
+        <v>0.4922848163736673</v>
+      </c>
+      <c r="H473" t="n">
+        <v>0.5033421329724079</v>
+      </c>
+      <c r="I473" t="n">
+        <v>10.22972460439459</v>
+      </c>
+      <c r="J473" t="n">
+        <v>0.0007850251894166065</v>
+      </c>
+      <c r="K473" t="n">
+        <v>11.27348794497099</v>
+      </c>
+      <c r="L473" t="n">
+        <v>0.7927354166666666</v>
+      </c>
+      <c r="M473" t="n">
+        <v>13.89473604166667</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C474" t="n">
+        <v>0.4678841188596546</v>
+      </c>
+      <c r="D474" t="n">
+        <v>2.137281347435427</v>
+      </c>
+      <c r="E474" t="n">
+        <v>0.5883871407502882</v>
+      </c>
+      <c r="F474" t="n">
+        <v>0.4591705416013628</v>
+      </c>
+      <c r="G474" t="n">
+        <v>0.363067353295966</v>
+      </c>
+      <c r="H474" t="n">
+        <v>0.3855931908863293</v>
+      </c>
+      <c r="I474" t="n">
+        <v>10.99234509453896</v>
+      </c>
+      <c r="J474" t="n">
+        <v>0.00107564018296657</v>
+      </c>
+      <c r="K474" t="n">
+        <v>11.2175047062077</v>
+      </c>
+      <c r="L474" t="n">
+        <v>0.7910354166666668</v>
+      </c>
+      <c r="M474" t="n">
+        <v>13.93548604166667</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B475" s="2" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C475" t="n">
+        <v>0.3155616454464329</v>
+      </c>
+      <c r="D475" t="n">
+        <v>3.168952927043067</v>
+      </c>
+      <c r="E475" t="n">
+        <v>0.398528104635988</v>
+      </c>
+      <c r="F475" t="n">
+        <v>0.72301368220492</v>
+      </c>
+      <c r="G475" t="n">
+        <v>0.3480676802068453</v>
+      </c>
+      <c r="H475" t="n">
+        <v>0.3754533879210153</v>
+      </c>
+      <c r="I475" t="n">
+        <v>7.425610149353222</v>
+      </c>
+      <c r="J475" t="n">
+        <v>0.00138698145525</v>
+      </c>
+      <c r="K475" t="n">
+        <v>11.2208937708823</v>
+      </c>
+      <c r="L475" t="n">
+        <v>0.8399104166666665</v>
+      </c>
+      <c r="M475" t="n">
+        <v>13.92306284722222</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="n">
+        <v>46072</v>
+      </c>
+      <c r="C476" t="n">
+        <v>0.4868000999168995</v>
+      </c>
+      <c r="D476" t="n">
+        <v>2.05423129570168</v>
+      </c>
+      <c r="E476" t="n">
+        <v>0.6099696014494087</v>
+      </c>
+      <c r="F476" t="n">
+        <v>0.4234785807330881</v>
+      </c>
+      <c r="G476" t="n">
+        <v>0.3890416322816693</v>
+      </c>
+      <c r="H476" t="n">
+        <v>0.3942181647749295</v>
+      </c>
+      <c r="I476" t="n">
+        <v>11.43684134939364</v>
+      </c>
+      <c r="J476" t="n">
+        <v>0.001255484551623328</v>
+      </c>
+      <c r="K476" t="n">
+        <v>11.26012334697547</v>
+      </c>
+      <c r="L476" t="n">
+        <v>0.8097569444444445</v>
+      </c>
+      <c r="M476" t="n">
+        <v>13.74050166666667</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B477" s="2" t="n">
+        <v>46073</v>
+      </c>
+      <c r="C477" t="n">
+        <v>0.3190796154659617</v>
+      </c>
+      <c r="D477" t="n">
+        <v>3.13401405645945</v>
+      </c>
+      <c r="E477" t="n">
+        <v>0.4381151251391347</v>
+      </c>
+      <c r="F477" t="n">
+        <v>0.7867258220417648</v>
+      </c>
+      <c r="G477" t="n">
+        <v>0.1441457610768002</v>
+      </c>
+      <c r="H477" t="n">
+        <v>0.1849025323969116</v>
+      </c>
+      <c r="I477" t="n">
+        <v>7.581143173248453</v>
+      </c>
+      <c r="J477" t="n">
+        <v>0.003127188955440007</v>
+      </c>
+      <c r="K477" t="n">
+        <v>11.01178147973113</v>
+      </c>
+      <c r="L477" t="n">
+        <v>0.8559896739130434</v>
+      </c>
+      <c r="M477" t="n">
+        <v>13.37822858997585</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B478" s="2" t="n">
+        <v>46074</v>
+      </c>
+      <c r="C478" t="n">
+        <v>0.9048237114080704</v>
+      </c>
+      <c r="D478" t="n">
+        <v>1.10518765964236</v>
+      </c>
+      <c r="E478" t="n">
+        <v>0.9161182608123229</v>
+      </c>
+      <c r="F478" t="n">
+        <v>0.04400828560345435</v>
+      </c>
+      <c r="G478" t="n">
+        <v>0.9245835190357808</v>
+      </c>
+      <c r="H478" t="n">
+        <v>0.9630138927885656</v>
+      </c>
+      <c r="I478" t="n">
+        <v>20.83444144559082</v>
+      </c>
+      <c r="J478" t="n">
+        <v>0.0006397043526666065</v>
+      </c>
+      <c r="K478" t="n">
+        <v>11.47118033467045</v>
+      </c>
+      <c r="L478" t="n">
+        <v>0.7737305555555555</v>
+      </c>
+      <c r="M478" t="n">
+        <v>13.55099951388889</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B479" s="2" t="n">
+        <v>46075</v>
+      </c>
+      <c r="C479" t="n">
+        <v>0.9661673896647306</v>
+      </c>
+      <c r="D479" t="n">
+        <v>1.035017338296845</v>
+      </c>
+      <c r="E479" t="n">
+        <v>0.9736868139856074</v>
+      </c>
+      <c r="F479" t="n">
+        <v>0.02464327136775467</v>
+      </c>
+      <c r="G479" t="n">
+        <v>0.9509959660722896</v>
+      </c>
+      <c r="H479" t="n">
+        <v>1.002885067009471</v>
+      </c>
+      <c r="I479" t="n">
+        <v>22.19349445861402</v>
+      </c>
+      <c r="J479" t="n">
+        <v>0.0006225079121666065</v>
+      </c>
+      <c r="K479" t="n">
+        <v>11.18133786904067</v>
+      </c>
+      <c r="L479" t="n">
+        <v>0.7702097222222223</v>
+      </c>
+      <c r="M479" t="n">
+        <v>14.45051097222222</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B480" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C480" t="n">
+        <v>0.3556171816060673</v>
+      </c>
+      <c r="D480" t="n">
+        <v>2.812012612786926</v>
+      </c>
+      <c r="E480" t="n">
+        <v>0.4964647051387568</v>
+      </c>
+      <c r="F480" t="n">
+        <v>0.8278793756589516</v>
+      </c>
+      <c r="G480" t="n">
+        <v>0.1501587652767687</v>
+      </c>
+      <c r="H480" t="n">
+        <v>0.1488970590971371</v>
+      </c>
+      <c r="I480" t="n">
+        <v>8.465587547636053</v>
+      </c>
+      <c r="J480" t="n">
+        <v>0.003065575607634834</v>
+      </c>
+      <c r="K480" t="n">
+        <v>10.90357556010304</v>
+      </c>
+      <c r="L480" t="n">
+        <v>0.8046637077294686</v>
+      </c>
+      <c r="M480" t="n">
+        <v>13.32683974637681</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B481" s="2" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C481" t="n">
+        <v>0.3063761974659914</v>
+      </c>
+      <c r="D481" t="n">
+        <v>3.26396113102423</v>
+      </c>
+      <c r="E481" t="n">
+        <v>0.3960089289536775</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0.6602980306938006</v>
+      </c>
+      <c r="G481" t="n">
+        <v>0.3074837403194067</v>
+      </c>
+      <c r="H481" t="n">
+        <v>0.3209794658581747</v>
+      </c>
+      <c r="I481" t="n">
+        <v>7.232496298943693</v>
+      </c>
+      <c r="J481" t="n">
+        <v>0.001507870410756686</v>
+      </c>
+      <c r="K481" t="n">
+        <v>11.26771868318409</v>
+      </c>
+      <c r="L481" t="n">
+        <v>0.8306159722222223</v>
+      </c>
+      <c r="M481" t="n">
+        <v>13.94483229166667</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B482" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="C482" t="n">
+        <v>0.4945657662849167</v>
+      </c>
+      <c r="D482" t="n">
+        <v>2.021975777886546</v>
+      </c>
+      <c r="E482" t="n">
+        <v>0.6069704268296039</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0.3548137795556159</v>
+      </c>
+      <c r="G482" t="n">
+        <v>0.3724911159196636</v>
+      </c>
+      <c r="H482" t="n">
+        <v>0.4444309529289005</v>
+      </c>
+      <c r="I482" t="n">
+        <v>11.61130026154466</v>
+      </c>
+      <c r="J482" t="n">
+        <v>0.001364495108299964</v>
+      </c>
+      <c r="K482" t="n">
+        <v>11.27673803272951</v>
+      </c>
+      <c r="L482" t="n">
+        <v>0.8657423611111111</v>
+      </c>
+      <c r="M482" t="n">
+        <v>14.05803618055555</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B483" s="2" t="n">
+        <v>46079</v>
+      </c>
+      <c r="C483" t="n">
+        <v>0.4408007891764758</v>
+      </c>
+      <c r="D483" t="n">
+        <v>2.268598479300016</v>
+      </c>
+      <c r="E483" t="n">
+        <v>0.5351425929790053</v>
+      </c>
+      <c r="F483" t="n">
+        <v>0.4940166513091905</v>
+      </c>
+      <c r="G483" t="n">
+        <v>0.4581675043785774</v>
+      </c>
+      <c r="H483" t="n">
+        <v>0.4711215008469862</v>
+      </c>
+      <c r="I483" t="n">
+        <v>10.33059809878521</v>
+      </c>
+      <c r="J483" t="n">
+        <v>0.001373721358403415</v>
+      </c>
+      <c r="K483" t="n">
+        <v>11.41725472163859</v>
+      </c>
+      <c r="L483" t="n">
+        <v>0.8546346618357488</v>
+      </c>
+      <c r="M483" t="n">
+        <v>13.76006088466183</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B484" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="C484" t="n">
+        <v>0.3195095967831071</v>
+      </c>
+      <c r="D484" t="n">
+        <v>3.129796444514405</v>
+      </c>
+      <c r="E484" t="n">
+        <v>0.432023477946169</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0.6462939643443389</v>
+      </c>
+      <c r="G484" t="n">
+        <v>0.3346354292747817</v>
+      </c>
+      <c r="H484" t="n">
+        <v>0.2186960646355338</v>
+      </c>
+      <c r="I484" t="n">
+        <v>7.589883955881267</v>
+      </c>
+      <c r="J484" t="n">
+        <v>0.003351765898446693</v>
+      </c>
+      <c r="K484" t="n">
+        <v>11.1069968383016</v>
+      </c>
+      <c r="L484" t="n">
+        <v>0.894488888888889</v>
+      </c>
+      <c r="M484" t="n">
+        <v>13.40249826388889</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B485" s="2" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C485" t="n">
+        <v>0.9256666961799407</v>
+      </c>
+      <c r="D485" t="n">
+        <v>1.080302450252147</v>
+      </c>
+      <c r="E485" t="n">
+        <v>0.9220581559064741</v>
+      </c>
+      <c r="F485" t="n">
+        <v>0.03093439705993986</v>
+      </c>
+      <c r="G485" t="n">
+        <v>0.9494300038892123</v>
+      </c>
+      <c r="H485" t="n">
+        <v>1.011740713696911</v>
+      </c>
+      <c r="I485" t="n">
+        <v>21.27635795781871</v>
+      </c>
+      <c r="J485" t="n">
+        <v>0.0007926653569166064</v>
+      </c>
+      <c r="K485" t="n">
+        <v>11.56486760224851</v>
+      </c>
+      <c r="L485" t="n">
+        <v>0.8220861111111111</v>
+      </c>
+      <c r="M485" t="n">
+        <v>13.55028631944444</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B486" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C486" t="n">
+        <v>0.956790646512984</v>
+      </c>
+      <c r="D486" t="n">
+        <v>1.045160718956119</v>
+      </c>
+      <c r="E486" t="n">
+        <v>0.9580450713954215</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0.0262956880578353</v>
+      </c>
+      <c r="G486" t="n">
+        <v>0.9560444202859775</v>
+      </c>
+      <c r="H486" t="n">
+        <v>0.99607192316972</v>
+      </c>
+      <c r="I486" t="n">
+        <v>21.97075378023377</v>
+      </c>
+      <c r="J486" t="n">
+        <v>0.00078998119225</v>
+      </c>
+      <c r="K486" t="n">
+        <v>11.63118863066726</v>
+      </c>
+      <c r="L486" t="n">
+        <v>0.8216034722222222</v>
+      </c>
+      <c r="M486" t="n">
+        <v>13.26433935897436</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B487" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="C487" t="n">
+        <v>0.4044707981811914</v>
+      </c>
+      <c r="D487" t="n">
+        <v>2.472366372298721</v>
+      </c>
+      <c r="E487" t="n">
+        <v>0.4516487541860671</v>
+      </c>
+      <c r="F487" t="n">
+        <v>0.418841417679449</v>
+      </c>
+      <c r="G487" t="n">
+        <v>0.6799908972209364</v>
+      </c>
+      <c r="H487" t="n">
+        <v>0.6866284547387037</v>
+      </c>
+      <c r="I487" t="n">
+        <v>9.344313478598815</v>
+      </c>
+      <c r="J487" t="n">
+        <v>0.00102943176391818</v>
+      </c>
+      <c r="K487" t="n">
+        <v>11.55647263754049</v>
+      </c>
+      <c r="L487" t="n">
+        <v>0.8488023912756483</v>
+      </c>
+      <c r="M487" t="n">
+        <v>13.56655911073651</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B488" s="2" t="n">
+        <v>46084</v>
+      </c>
+      <c r="C488" t="n">
+        <v>0.4325658695936999</v>
+      </c>
+      <c r="D488" t="n">
+        <v>2.311786644053261</v>
+      </c>
+      <c r="E488" t="n">
+        <v>0.5422324752240214</v>
+      </c>
+      <c r="F488" t="n">
+        <v>0.4242116185694415</v>
+      </c>
+      <c r="G488" t="n">
+        <v>0.3534344614026845</v>
+      </c>
+      <c r="H488" t="n">
+        <v>0.393249515800323</v>
+      </c>
+      <c r="I488" t="n">
+        <v>10.13130487235824</v>
+      </c>
+      <c r="J488" t="n">
+        <v>0.001833273495059515</v>
+      </c>
+      <c r="K488" t="n">
+        <v>11.33434554485194</v>
+      </c>
+      <c r="L488" t="n">
+        <v>0.9007003485879358</v>
+      </c>
+      <c r="M488" t="n">
+        <v>13.99632091549362</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B489" s="2" t="n">
+        <v>46085</v>
+      </c>
+      <c r="C489" t="n">
+        <v>0.512877520214177</v>
+      </c>
+      <c r="D489" t="n">
+        <v>1.949783253480093</v>
+      </c>
+      <c r="E489" t="n">
+        <v>0.6064506328738862</v>
+      </c>
+      <c r="F489" t="n">
+        <v>0.3420985255969076</v>
+      </c>
+      <c r="G489" t="n">
+        <v>0.4763229234352562</v>
+      </c>
+      <c r="H489" t="n">
+        <v>0.5371109818966843</v>
+      </c>
+      <c r="I489" t="n">
+        <v>11.93584715259641</v>
+      </c>
+      <c r="J489" t="n">
+        <v>0.002064588836277998</v>
+      </c>
+      <c r="K489" t="n">
+        <v>11.19010846795876</v>
+      </c>
+      <c r="L489" t="n">
+        <v>0.915687004758967</v>
+      </c>
+      <c r="M489" t="n">
+        <v>14.07044806197982</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B490" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="C490" t="n">
+        <v>0.4918548444608812</v>
+      </c>
+      <c r="D490" t="n">
+        <v>2.033120159863614</v>
+      </c>
+      <c r="E490" t="n">
+        <v>0.5116508752535788</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0.4871099175221535</v>
+      </c>
+      <c r="G490" t="n">
+        <v>0.305271560189486</v>
+      </c>
+      <c r="H490" t="n">
+        <v>0.8839284847335409</v>
+      </c>
+      <c r="I490" t="n">
+        <v>11.42871844800069</v>
+      </c>
+      <c r="J490" t="n">
+        <v>0.001525386699947776</v>
+      </c>
+      <c r="K490" t="n">
+        <v>11.0717313735033</v>
+      </c>
+      <c r="L490" t="n">
+        <v>0.8863414537280428</v>
+      </c>
+      <c r="M490" t="n">
+        <v>14.28657196094448</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B491" s="2" t="n">
+        <v>46087</v>
+      </c>
+      <c r="C491" t="n">
+        <v>0.3143554283690782</v>
+      </c>
+      <c r="D491" t="n">
+        <v>3.181112555263148</v>
+      </c>
+      <c r="E491" t="n">
+        <v>0.4473722121348514</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0.8498243676530033</v>
+      </c>
+      <c r="G491" t="n">
+        <v>0.1090496793337675</v>
+      </c>
+      <c r="H491" t="n">
+        <v>0.108012655964797</v>
+      </c>
+      <c r="I491" t="n">
+        <v>7.49738960377904</v>
+      </c>
+      <c r="J491" t="n">
+        <v>0.003280234945084576</v>
+      </c>
+      <c r="K491" t="n">
+        <v>10.82681702414147</v>
+      </c>
+      <c r="L491" t="n">
+        <v>0.8116596480754653</v>
+      </c>
+      <c r="M491" t="n">
+        <v>13.79904621321637</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B492" s="2" t="n">
+        <v>46088</v>
+      </c>
+      <c r="C492" t="n">
+        <v>0.8534719736858385</v>
+      </c>
+      <c r="D492" t="n">
+        <v>1.171684637377558</v>
+      </c>
+      <c r="E492" t="n">
+        <v>0.9383279774408607</v>
+      </c>
+      <c r="F492" t="n">
+        <v>0.09543178382068931</v>
+      </c>
+      <c r="G492" t="n">
+        <v>0.7521186529562675</v>
+      </c>
+      <c r="H492" t="n">
+        <v>0.7287003932682896</v>
+      </c>
+      <c r="I492" t="n">
+        <v>19.68656247723694</v>
+      </c>
+      <c r="J492" t="n">
+        <v>0.0007120088373756656</v>
+      </c>
+      <c r="K492" t="n">
+        <v>11.39908057526985</v>
+      </c>
+      <c r="L492" t="n">
+        <v>0.7983819660307975</v>
+      </c>
+      <c r="M492" t="n">
+        <v>13.81141102308535</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B493" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C493" t="n">
+        <v>0.9771667290766332</v>
+      </c>
+      <c r="D493" t="n">
+        <v>1.023366811664723</v>
+      </c>
+      <c r="E493" t="n">
+        <v>0.9809604938468649</v>
+      </c>
+      <c r="F493" t="n">
+        <v>0.01154857173559073</v>
+      </c>
+      <c r="G493" t="n">
+        <v>0.9780052105391224</v>
+      </c>
+      <c r="H493" t="n">
+        <v>0.9956995631477249</v>
+      </c>
+      <c r="I493" t="n">
+        <v>22.47724631685945</v>
+      </c>
+      <c r="J493" t="n">
+        <v>0.000817377064790053</v>
+      </c>
+      <c r="K493" t="n">
+        <v>11.3655393474548</v>
+      </c>
+      <c r="L493" t="n">
+        <v>0.8235746325997481</v>
+      </c>
+      <c r="M493" t="n">
+        <v>13.77018424033798</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B494" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C494" t="n">
+        <v>0.340967722655133</v>
+      </c>
+      <c r="D494" t="n">
+        <v>2.93282892648298</v>
+      </c>
+      <c r="E494" t="n">
+        <v>0.3928311447807619</v>
+      </c>
+      <c r="F494" t="n">
+        <v>0.6517708073089044</v>
+      </c>
+      <c r="G494" t="n">
+        <v>0.4760681317625114</v>
+      </c>
+      <c r="H494" t="n">
+        <v>0.6039258382536815</v>
+      </c>
+      <c r="I494" t="n">
+        <v>7.948025997995789</v>
+      </c>
+      <c r="J494" t="n">
+        <v>0.001139731559475576</v>
+      </c>
+      <c r="K494" t="n">
+        <v>11.16805849583465</v>
+      </c>
+      <c r="L494" t="n">
+        <v>0.8354524101188402</v>
+      </c>
+      <c r="M494" t="n">
+        <v>14.12087006324119</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B495" s="2" t="n">
+        <v>46091</v>
+      </c>
+      <c r="C495" t="n">
+        <v>0.3140325988283595</v>
+      </c>
+      <c r="D495" t="n">
+        <v>3.184382779784494</v>
+      </c>
+      <c r="E495" t="n">
+        <v>0.4339089044673531</v>
+      </c>
+      <c r="F495" t="n">
+        <v>0.8068303361112311</v>
+      </c>
+      <c r="G495" t="n">
+        <v>0.1472736884929488</v>
+      </c>
+      <c r="H495" t="n">
+        <v>0.1711879769822992</v>
+      </c>
+      <c r="I495" t="n">
+        <v>7.457119628653643</v>
+      </c>
+      <c r="J495" t="n">
+        <v>0.003209546534094031</v>
+      </c>
+      <c r="K495" t="n">
+        <v>10.87534063723062</v>
+      </c>
+      <c r="L495" t="n">
+        <v>0.8395768066326229</v>
+      </c>
+      <c r="M495" t="n">
+        <v>13.74146343665395</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B496" s="2" t="n">
+        <v>46092</v>
+      </c>
+      <c r="C496" t="n">
+        <v>0.5623868861152572</v>
+      </c>
+      <c r="D496" t="n">
+        <v>1.778135345416033</v>
+      </c>
+      <c r="E496" t="n">
+        <v>0.6867859294878046</v>
+      </c>
+      <c r="F496" t="n">
+        <v>0.2801749420478789</v>
+      </c>
+      <c r="G496" t="n">
+        <v>0.4772305306453725</v>
+      </c>
+      <c r="H496" t="n">
+        <v>0.4566034129499895</v>
+      </c>
+      <c r="I496" t="n">
+        <v>13.19637772810084</v>
+      </c>
+      <c r="J496" t="n">
+        <v>0.001612127670929551</v>
+      </c>
+      <c r="K496" t="n">
+        <v>11.21185640103508</v>
+      </c>
+      <c r="L496" t="n">
+        <v>0.8674239076870179</v>
+      </c>
+      <c r="M496" t="n">
+        <v>14.18510708006051</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>SmartMeter_SM_ECOVILLA</t>
+        </is>
+      </c>
+      <c r="B497" s="2" t="n">
+        <v>46093</v>
+      </c>
+      <c r="C497" t="n">
+        <v>0.478620267436445</v>
+      </c>
+      <c r="D497" t="n">
+        <v>2.08933901891814</v>
+      </c>
+      <c r="E497" t="n">
+        <v>0.6380660106006206</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0.3849093146344444</v>
+      </c>
+      <c r="G497" t="n">
+        <v>0.252463111543049</v>
+      </c>
+      <c r="H497" t="n">
+        <v>0.2503326904339239</v>
+      </c>
+      <c r="I497" t="n">
+        <v>8.271295711696919</v>
+      </c>
+      <c r="J497" t="n">
+        <v>0.001317429202091078</v>
+      </c>
+      <c r="K497" t="n">
+        <v>11.18064755236801</v>
+      </c>
+      <c r="L497" t="n">
+        <v>0.8333184302105594</v>
+      </c>
+      <c r="M497" t="n">
+        <v>14.08478207173526</v>
       </c>
     </row>
   </sheetData>

</xml_diff>